<commit_message>
import notebook pipeline28 code config and global handoff
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11610" yWindow="1590" windowWidth="13590" windowHeight="11790" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mappings" sheetId="1" state="visible" r:id="rId1"/>
@@ -35,15 +35,21 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.5999938962981048"/>
+        <bgColor theme="4" tint="0.5999938962981048"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -66,15 +72,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,12 +560,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Potência Total_mean_mean_of_windows</t>
+          <t>Potência Total_mean_of_windows</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Potência Total_mean_sd_of_windows</t>
+          <t>Potência Total_sd_of_windows</t>
         </is>
       </c>
     </row>
@@ -584,12 +606,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T_CARTER_mean_mean_of_windows</t>
+          <t>T_CARTER_mean_of_windows</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>T_CARTER_mean_sd_of_windows</t>
+          <t>T_CARTER_sd_of_windows</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -606,12 +628,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T_AMBIENTE_mean_mean_of_windows</t>
+          <t>T_AMBIENTE_mean_of_windows</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>T_AMBIENTE_mean_sd_of_windows</t>
+          <t>T_AMBIENTE_sd_of_windows</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -635,6 +657,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="68.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="66" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="72.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="66" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="66.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="62.28515625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="56.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="61.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="71.7109375" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="78.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="36.42578125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="58.140625" bestFit="1" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1348,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:T42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1357,15 +1390,9 @@
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="7" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="10" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="36" customWidth="1" min="18" max="18"/>
@@ -1449,15 +1476,25 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>y_tol_plus</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>y_tol_minus</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>filter_h2o_list</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>label_variant</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -1525,12 +1562,18 @@
       <c r="O2" t="n">
         <v>2</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Legacy: nth with error bars</t>
         </is>
@@ -1589,12 +1632,18 @@
       <c r="L3" t="n">
         <v>5</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Legacy: consumo with error bars</t>
         </is>
@@ -1648,12 +1697,18 @@
       <c r="L4" t="n">
         <v>5</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Legacy: MFB_10_90</t>
         </is>
@@ -1707,12 +1762,18 @@
       <c r="L5" t="n">
         <v>5</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Legacy: Delta-T no labels</t>
         </is>
@@ -1766,17 +1827,23 @@
       <c r="L6" t="n">
         <v>5</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>box</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Legacy: labels box</t>
         </is>
@@ -1830,17 +1897,23 @@
       <c r="L7" t="n">
         <v>5</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Legacy: labels tag</t>
         </is>
@@ -1894,17 +1967,23 @@
       <c r="L8" t="n">
         <v>5</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>marker</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Legacy: labels marker</t>
         </is>
@@ -1958,17 +2037,23 @@
       <c r="L9" t="n">
         <v>5</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>badge</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Legacy: labels badge</t>
         </is>
@@ -2022,12 +2107,18 @@
       <c r="L10" t="n">
         <v>5</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Legacy: Air_kg_h</t>
         </is>
@@ -2081,12 +2172,18 @@
       <c r="L11" t="n">
         <v>5</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Legacy: Air_g_s</t>
         </is>
@@ -2140,12 +2237,18 @@
       <c r="L12" t="n">
         <v>5</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Legacy: humidity</t>
         </is>
@@ -2199,12 +2302,18 @@
       <c r="L13" t="n">
         <v>5</v>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Legacy: T_E_CIL_AVG</t>
         </is>
@@ -2258,12 +2367,18 @@
       <c r="L14" t="n">
         <v>5</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Legacy: Q_EVAP_NET vs power</t>
         </is>
@@ -2308,12 +2423,18 @@
           <t>Q_EVAP_NET (kW)</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Legacy: Q_EVAP_NET vs Air_kg_h</t>
         </is>
@@ -2340,7 +2461,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>P_COLETOR_RAW_mean_mean_of_windows</t>
+          <t>P_COLETOR_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2358,12 +2479,18 @@
           <t>Q_EVAP_NET (kW)</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>Legacy: Q_EVAP_NET vs P_COLETOR (will skip if col missing)</t>
         </is>
@@ -2380,7 +2507,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>raw_P_E_TURB_RAW_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_P_E_TURB_RAW_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2395,7 +2522,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>P_E_TURB_RAW_mean_mean_of_windows</t>
+          <t>P_E_TURB_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2417,12 +2544,18 @@
       <c r="L17" t="n">
         <v>5</v>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2439,7 +2572,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>raw_P_S_TURB_RAW_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_P_S_TURB_RAW_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2454,7 +2587,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>P_S_TURB_RAW_mean_mean_of_windows</t>
+          <t>P_S_TURB_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2476,12 +2609,18 @@
       <c r="L18" t="n">
         <v>5</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2498,7 +2637,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>raw_P_E_COMP_RAW_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_P_E_COMP_RAW_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2513,7 +2652,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>P_E_COMP_RAW_mean_mean_of_windows</t>
+          <t>P_E_COMP_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2535,12 +2674,18 @@
       <c r="L19" t="n">
         <v>5</v>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2557,7 +2702,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>raw_P_S_COMP_RAW_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_P_S_COMP_RAW_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2572,7 +2717,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>P_S_COMP_RAW_mean_mean_of_windows</t>
+          <t>P_S_COMP_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2594,12 +2739,18 @@
       <c r="L20" t="n">
         <v>5</v>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2616,7 +2767,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>raw_P_COLETOR_RAW_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_P_COLETOR_RAW_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2631,7 +2782,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>P_COLETOR_RAW_mean_mean_of_windows</t>
+          <t>P_COLETOR_RAW_mean_of_windows</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2653,12 +2804,18 @@
       <c r="L21" t="n">
         <v>5</v>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2675,7 +2832,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>raw_T_ADMISS_O_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_ADMISS_O_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2690,7 +2847,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>T_ADMISSÃO_mean_mean_of_windows</t>
+          <t>T_ADMISSÃO_mean_of_windows</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2712,12 +2869,18 @@
       <c r="L22" t="n">
         <v>5</v>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2734,7 +2897,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>raw_T_E_TURB_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_TURB_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2749,7 +2912,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>T_E_TURB_mean_mean_of_windows</t>
+          <t>T_E_TURB_mean_of_windows</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2771,12 +2934,18 @@
       <c r="L23" t="n">
         <v>5</v>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2793,7 +2962,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>raw_T_S_TURB_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_S_TURB_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2808,7 +2977,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>T_S_TURB_mean_mean_of_windows</t>
+          <t>T_S_TURB_mean_of_windows</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2830,12 +2999,18 @@
       <c r="L24" t="n">
         <v>5</v>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2852,7 +3027,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>raw_T_E_COMP_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_COMP_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2867,7 +3042,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>T_E_COMP_mean_mean_of_windows</t>
+          <t>T_E_COMP_mean_of_windows</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2889,12 +3064,18 @@
       <c r="L25" t="n">
         <v>5</v>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2911,7 +3092,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>raw_T_S_COMP_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_S_COMP_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2926,7 +3107,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>T_S_COMP_mean_mean_of_windows</t>
+          <t>T_S_COMP_mean_of_windows</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2948,12 +3129,18 @@
       <c r="L26" t="n">
         <v>5</v>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -2970,7 +3157,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>raw_T_E_CIL_1_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_CIL_1_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2985,7 +3172,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>T_S_CIL_1_mean_mean_of_windows</t>
+          <t>T_S_CIL_1_mean_of_windows</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3007,12 +3194,18 @@
       <c r="L27" t="n">
         <v>5</v>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -3029,7 +3222,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>raw_T_E_CIL_2_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_CIL_2_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3044,7 +3237,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>T_S_CIL_2_mean_mean_of_windows</t>
+          <t>T_S_CIL_2_mean_of_windows</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3066,12 +3259,18 @@
       <c r="L28" t="n">
         <v>5</v>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -3088,7 +3287,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>raw_T_E_CIL_3_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_CIL_3_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3103,7 +3302,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>T_S_CIL_3_mean_mean_of_windows</t>
+          <t>T_S_CIL_3_mean_of_windows</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3125,12 +3324,18 @@
       <c r="L29" t="n">
         <v>5</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -3147,7 +3352,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>raw_T_E_CIL_4_mean_mean_of_windows_vs_power_all.png</t>
+          <t>raw_T_E_CIL_4_mean_of_windows_vs_power_all.png</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3162,7 +3367,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>T_S_CIL_4_mean_mean_of_windows</t>
+          <t>T_S_CIL_4_mean_of_windows</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3184,12 +3389,18 @@
       <c r="L30" t="n">
         <v>5</v>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>Legacy: raw requested list</t>
         </is>
@@ -3233,14 +3444,763 @@
       <c r="L31" t="n">
         <v>5</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="inlineStr">
         <is>
           <t>6,25,35</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="T31" t="inlineStr">
         <is>
           <t>AUTO: expand one plot per KIBOX_* column (except KIBOX_N_files)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nox_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>NOX vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NOX_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>NOX</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>55</v>
+      </c>
+      <c r="L32" t="n">
+        <v>5</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Added: gas emissions via config (NOX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>co_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CO vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CO_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>55</v>
+      </c>
+      <c r="L33" t="n">
+        <v>5</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Added: gas emissions via config (CO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>co2_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CO2 vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>CO2_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>55</v>
+      </c>
+      <c r="L34" t="n">
+        <v>5</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Added: gas emissions via config (CO2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>o2_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>O2 vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>O2_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>55</v>
+      </c>
+      <c r="L35" t="n">
+        <v>5</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Added: gas emissions via config (O2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ect_ctrl_error_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ECT control error (T_S_AGUA - DEM_TH2O) vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>ECT_CTRL_ERROR_C</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Control error (degC)</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>55</v>
+      </c>
+      <c r="L36" t="n">
+        <v>5</v>
+      </c>
+      <c r="M36" t="n">
+        <v>-10</v>
+      </c>
+      <c r="N36" t="n">
+        <v>10</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>ECT control stability with +/-2C tolerance</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>bsfc_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Specific fuel consumption vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BSFC_g_kWh</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>U_BSFC_g_kWh</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Specific fuel consumption (g/kWh)</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>55</v>
+      </c>
+      <c r="L37" t="n">
+        <v>5</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>BSFC from Consumo_kg_h and power with propagated uncertainty from fuel and power channels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>t_s_agua_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Engine Coolant temperature vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>T_S_AGUA_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Temperature (°C)</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>55</v>
+      </c>
+      <c r="L38" t="n">
+        <v>5</v>
+      </c>
+      <c r="M38" t="n">
+        <v>80</v>
+      </c>
+      <c r="N38" t="n">
+        <v>90</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>-87</v>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>t_watercooler_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>T_WATERCOOLER vs Load (all fuels)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>T_WATERCOOLER_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Power command (kW)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>T_WATERCOOLER (degC)</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>55</v>
+      </c>
+      <c r="L39" t="n">
+        <v>5</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Added by request: temperature vs Load_kW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>t_radiador_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>T_RADIADOR vs Load (all fuels)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>T_RADIADOR_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Power command (kW)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>T_RADIADOR (degC)</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>55</v>
+      </c>
+      <c r="L40" t="n">
+        <v>5</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Added by request: temperature vs Load_kW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>t_carter_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>T_CARTER vs Load (all fuels)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>T_CARTER_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Power command (kW)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>T_CARTER (degC)</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>55</v>
+      </c>
+      <c r="L41" t="n">
+        <v>5</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Added by request: temperature vs Load_kW with uncertainty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>t_ambiente_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>T_AMBIENTE vs Load (all fuels)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>T_AMBIENTE_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Power command (kW)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>T_AMBIENTE (degC)</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>55</v>
+      </c>
+      <c r="L42" t="n">
+        <v>5</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Added by request: temperature vs Load_kW with uncertainty.</t>
         </is>
       </c>
     </row>
@@ -3258,7 +4218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3329,6 +4289,26 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MAX_ECT_CONTROL_ERROR</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>degC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Erro de controle se |T_S_AGUA - DEM_TH2O| exceder este limite (faixa +-2 degC).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add configurable raw input and output directories
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -171,6 +171,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Codex</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Diretorio varrido recursivamente para ler os arquivos LabVIEW/Kibox. Se vazio, usa raw\PROCESSAR ao lado do script. Aceita caminho absoluto ou relativo ao diretorio do script.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>Diretorio de saida do pipeline. Se vazio, usa out ao lado do script. Aceita caminho absoluto ou relativo ao diretorio do script.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1307,7 +1327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1370,8 +1390,25 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RAW_INPUT_DIR</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OUT_DIR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
use sd uncertainty for motec lambda plot
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -4284,7 +4284,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>off</t>
+          <t>Motec_Exhaust Lambda_sd_of_windows</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Added by request: MoTeC exhaust lambda vs Load_kW with fixed lambda scale 0.90..1.10 step 0.02.</t>
+          <t>Added by request: MoTeC exhaust lambda vs Load_kW with SD-only uncertainty and fixed lambda scale 0.90..1.10 step 0.02.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add motec closed loop trim plot
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -1430,7 +1430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4399,6 +4399,76 @@
       <c r="T44" t="inlineStr">
         <is>
           <t>Added by request: MoTeC ignition advance vs Load_kW with SD-only uncertainty and autoscale on Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>motec_fuel_closed_loop_trim_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MoTeC fuel closed loop trim vs Load (all fuels)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Motec_Fuel Closed Loop Control Bank 1 Trim_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Motec_Fuel Closed Loop Control Bank 1 Trim_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Power command (kW)</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Fuel closed loop trim bank 1 (%Trim)</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>55</v>
+      </c>
+      <c r="L45" t="n">
+        <v>5</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>6,25,35</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Added by request: MoTeC fuel closed loop control bank 1 trim vs Load_kW with SD-only uncertainty and autoscale on Y.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
set ignition advance ticks to 1 degree
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -4385,6 +4385,9 @@
       <c r="L44" t="n">
         <v>5</v>
       </c>
+      <c r="O44" t="n">
+        <v>1</v>
+      </c>
       <c r="P44" t="n">
         <v>0</v>
       </c>
@@ -4398,7 +4401,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Added by request: MoTeC ignition advance vs Load_kW with SD-only uncertainty and autoscale on Y.</t>
+          <t>Added by request: MoTeC ignition advance vs Load_kW with SD-only uncertainty and autoscale on Y. Y ticks: 1 deg autoscale.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
enforce strict RAW/OUT dirs from Excel defaults in pipeline28
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\_tmp_nanum_pipeline_28_remote_20260309\raw\PROCESSAR</t>
+          <t>C:\Users\SC61730\Downloads\raw_mestrado</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\_tmp_nanum_pipeline_28_remote_20260309\out</t>
+          <t>C:\Users\SC61730\Downloads\out_mestrado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add ignition delay metric and UPD-power all-fuels plot
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -1430,7 +1430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4472,6 +4472,62 @@
       <c r="T45" t="inlineStr">
         <is>
           <t>Added by request: MoTeC fuel closed loop control bank 1 trim vs Load_kW with SD-only uncertainty and autoscale on Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ignition_delay_vs_upd_power_all.png</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Ignition delay (abs) vs UPD measured power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UPD_Power_Bin_kW</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Ignition_Delay_abs_degCA</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>off</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Potencia UPD medida (kW, bin 0.1)</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Ignition delay abs (deg CA)</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Added by request: abs(KIBOX_AI05_1 + Motec_Ignition Timing_mean_of_windows) with UPD power on X.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tune ignition-delay plot scales to match kibox x-axis and 0.5deg y ticks
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -4519,6 +4519,18 @@
           <t>Ignition delay abs (deg CA)</t>
         </is>
       </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>55</v>
+      </c>
+      <c r="L46" t="n">
+        <v>5</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.5</v>
+      </c>
       <c r="P46" t="n">
         <v>0</v>
       </c>
@@ -4527,7 +4539,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Added by request: abs(KIBOX_AI05_1 + Motec_Ignition Timing_mean_of_windows) with UPD power on X.</t>
+          <t>Added by request: abs(KIBOX_AI05_1 + Motec_Ignition Timing_mean_of_windows) with UPD power on X. | Y step set to 0.5 deg and X scale aligned with kibox (0..55 step 5).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add volumetric fuel flow and hourly cost outputs
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -1327,7 +1327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\raw_NANUM</t>
+          <t>C:\Users\SC61730\Downloads\raw_mestrado\raw</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,63 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\out_NANUM</t>
+          <t>C:\Users\SC61730\Downloads\out_mestrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FUEL_DENSITY_KG_M3_D85B15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FUEL_DENSITY_KG_M3_E94H6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FUEL_DENSITY_KG_M3_E75H25</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FUEL_DENSITY_KG_M3_E65H35</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FUEL_COST_R_L_D85B15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FUEL_COST_R_L_E94H6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FUEL_COST_R_L_E75H25</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FUEL_COST_R_L_E65H35</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T46"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4540,6 +4596,146 @@
       <c r="T46" t="inlineStr">
         <is>
           <t>Added by request: abs(KIBOX_AI05_1 + Motec_Ignition Timing_mean_of_windows) with UPD power on X. | Y step set to 0.5 deg and X scale aligned with kibox (0..55 step 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>consumo_l_h_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Volumetric fuel flow vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Consumo_L_h</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>U_Consumo_L_h</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Fuel flow (L/h)</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>55</v>
+      </c>
+      <c r="L47" t="n">
+        <v>5</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>0,6,25,35</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Fuel volumetric flow from kg/h and density in Defaults</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>custo_r_h_vs_power_all.png</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Fuel cost vs Power (all fuels)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Custo_R_h</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>U_Custo_R_h</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Fuel cost (R$/h)</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>55</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>0,6,25,35</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Fuel hourly cost from volumetric flow and cost in Defaults</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record pipeline28 diesel savings and scenario workflow
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="3" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="975" yWindow="240" windowWidth="21210" windowHeight="11295" tabRatio="600" firstSheet="3" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mappings" sheetId="1" state="visible" r:id="rId1"/>
@@ -1327,10 +1327,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="48.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="22" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1424,6 +1424,9 @@
           <t>FUEL_DENSITY_KG_M3_D85B15</t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>853</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1431,6 +1434,9 @@
           <t>FUEL_DENSITY_KG_M3_E94H6</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>809</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1438,6 +1444,9 @@
           <t>FUEL_DENSITY_KG_M3_E75H25</t>
         </is>
       </c>
+      <c r="B10" t="n">
+        <v>873</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1445,6 +1454,9 @@
           <t>FUEL_DENSITY_KG_M3_E65H35</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>897</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1452,6 +1464,9 @@
           <t>FUEL_COST_R_L_D85B15</t>
         </is>
       </c>
+      <c r="B12" t="n">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1459,6 +1474,9 @@
           <t>FUEL_COST_R_L_E94H6</t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1466,12 +1484,78 @@
           <t>FUEL_COST_R_L_E75H25</t>
         </is>
       </c>
+      <c r="B14" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>FUEL_COST_R_L_E65H35</t>
         </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MACHINE_HOURS_PER_YEAR_COLHEITADEIRA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MACHINE_DIESEL_L_H_COLHEITADEIRA</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MACHINE_HOURS_PER_YEAR_TRATOR_TRANSBORDO</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MACHINE_DIESEL_L_H_TRATOR_TRANSBORDO</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MACHINE_HOURS_PER_YEAR_CAMINHAO</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MACHINE_DIESEL_L_H_CAMINHAO</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1486,7 +1570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1675,7 +1759,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -1745,7 +1829,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1810,7 +1894,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1875,7 +1959,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1940,7 +2024,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -2010,7 +2094,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -2080,7 +2164,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2150,7 +2234,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -2220,7 +2304,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -2285,7 +2369,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -2350,7 +2434,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -2415,7 +2499,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2480,7 +2564,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2536,7 +2620,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2592,7 +2676,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2657,7 +2741,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2722,7 +2806,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2787,7 +2871,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2852,7 +2936,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2917,7 +3001,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2982,7 +3066,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -3047,7 +3131,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -3112,7 +3196,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -3177,7 +3261,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -3242,7 +3326,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -3307,7 +3391,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -3372,7 +3456,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -3437,7 +3521,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -3502,7 +3586,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -3557,7 +3641,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -3622,7 +3706,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3687,7 +3771,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -3752,7 +3836,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -3817,7 +3901,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -3891,7 +3975,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -3961,7 +4045,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -4035,7 +4119,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4179,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -4160,7 +4244,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4230,7 +4314,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
@@ -4300,7 +4384,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -4379,7 +4463,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
@@ -4452,7 +4536,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -4522,7 +4606,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>6,25,35</t>
+          <t>0,6,25,35</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
@@ -4736,6 +4820,146 @@
       <c r="T48" t="inlineStr">
         <is>
           <t>Fuel hourly cost from volumetric flow and cost in Defaults</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>economia_pct_vs_diesel_power_all.png</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Hourly cost delta vs Diesel vs Power (negative = saving)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Economia_vs_Diesel_pct</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>U_Economia_vs_Diesel_pct</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Cost delta vs Diesel (%)</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>55</v>
+      </c>
+      <c r="L49" t="n">
+        <v>5</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>0,6,25,35</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Signed hourly cost delta relative to diesel baseline. Negative values mean savings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>all_fuels_yx</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>economia_r_h_vs_diesel_power_all.png</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Hourly cost delta vs Diesel vs Power (negative = saving)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Load_kW</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Economia_vs_Diesel_R_h</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>U_Economia_vs_Diesel_R_h</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Power (kW)</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Cost delta vs Diesel (R$/h)</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>55</v>
+      </c>
+      <c r="L50" t="n">
+        <v>5</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>0,6,25,35</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Signed hourly cost delta relative to diesel baseline. Negative values mean savings.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pipeline29: consolidate Wagner fuels, airflow and emissions flow
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -9572,7 +9572,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\raw_mestrado</t>
+          <t>C:\Users\SC61730\Downloads\raw_wagnao</t>
         </is>
       </c>
     </row>
@@ -9584,7 +9584,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C:\Users\SC61730\Downloads\out_mestrado</t>
+          <t>C:\Users\SC61730\Downloads\out_wagnao</t>
         </is>
       </c>
     </row>

</xml_diff>